<commit_message>
Added another way to calculate the reference trajectory still needs tunning as well as updates MFEval library which still needs checks
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32436DAD-AE86-834A-96B0-C055C3929EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F3B4172-D12B-7E4D-870A-519C641D20C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3920" yWindow="1880" windowWidth="34480" windowHeight="19400" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -623,7 +623,7 @@
     <t>1 combined</t>
   </si>
   <si>
-    <t>which('Hoosier_R20B_20p5x7_R13_7in_v2.tir')</t>
+    <t>which('Hoosier_R20B_20p5x7_R13_7in_12psi.tir')</t>
   </si>
 </sst>
 </file>
@@ -7720,6 +7720,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7980,7 +7989,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
@@ -7991,16 +8000,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8019,7 +8027,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -8028,12 +8036,4 @@
     <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added agent skill for multiple simulations - still in testing
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE07DA8-DC25-5441-953A-F8DD93D1778D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77795C3B-A319-DE47-9FA4-D1F9D0FCB09C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3920" yWindow="1880" windowWidth="34480" windowHeight="19400" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7720,14 +7720,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7992,21 +7990,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8031,9 +8028,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>